<commit_message>
OO-9303: add rooms to the curriculum import/export
</commit_message>
<xml_diff>
--- a/src/main/java/org/olat/modules/curriculum/ui/importwizard/products-example.xlsx
+++ b/src/main/java/org/olat/modules/curriculum/ui/importwizard/products-example.xlsx
@@ -1,41 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srosse/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7B7DE7-158B-9648-B6D7-7D5B115982BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="860" yWindow="620" windowWidth="46600" windowHeight="22300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Implementations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Memberships" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Users" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Export Information" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Products" sheetId="1" r:id="rId1"/>
+    <sheet name="Implementations" sheetId="2" r:id="rId2"/>
+    <sheet name="Memberships" sheetId="3" r:id="rId3"/>
+    <sheet name="Users" sheetId="4" r:id="rId4"/>
+    <sheet name="Export Information" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Implementations!$A$1:$U$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Implementations!$A$1:$U$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Implementations!$A$1:$V$39</definedName>
   </definedNames>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
-  <si>
-    <t xml:space="preserve">Title *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ext. Ref. *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORG - Ext. Ref. *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Absences *</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="153">
+  <si>
+    <t>Title *</t>
+  </si>
+  <si>
+    <t>Ext. Ref. *</t>
+  </si>
+  <si>
+    <t>ORG - Ext. Ref. *</t>
+  </si>
+  <si>
+    <t>Absences *</t>
   </si>
   <si>
     <t>Description</t>
@@ -44,7 +47,7 @@
     <t xml:space="preserve">Creation Date </t>
   </si>
   <si>
-    <t xml:space="preserve">Last Modified</t>
+    <t>Last Modified</t>
   </si>
   <si>
     <t>Spanish</t>
@@ -59,19 +62,19 @@
     <t>OFF</t>
   </si>
   <si>
-    <t xml:space="preserve">1/12/2026, 3:21 PM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1/14/2026, 11:45 AM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROD - Ext. Ref. *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IMPL - Ext. Ref. *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Object Type *</t>
+    <t>1/12/2026, 3:21 PM</t>
+  </si>
+  <si>
+    <t>1/14/2026, 11:45 AM</t>
+  </si>
+  <si>
+    <t>PROD - Ext. Ref. *</t>
+  </si>
+  <si>
+    <t>IMPL - Ext. Ref. *</t>
+  </si>
+  <si>
+    <t>Object Type *</t>
   </si>
   <si>
     <t>Level</t>
@@ -80,28 +83,28 @@
     <t>Status</t>
   </si>
   <si>
-    <t xml:space="preserve">Date - Begin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Time - Begin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date - End</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Time - End</t>
+    <t>Date - Begin</t>
+  </si>
+  <si>
+    <t>Time - Begin</t>
+  </si>
+  <si>
+    <t>Date - End</t>
+  </si>
+  <si>
+    <t>Time - End</t>
   </si>
   <si>
     <t>Unit</t>
   </si>
   <si>
-    <t xml:space="preserve">REF - Ext. Ref.</t>
+    <t>REF - Ext. Ref.</t>
   </si>
   <si>
     <t>Location</t>
   </si>
   <si>
-    <t xml:space="preserve">ELEM Type - Ext. Ref.</t>
+    <t>ELEM Type - Ext. Ref.</t>
   </si>
   <si>
     <t>Calendar</t>
@@ -122,7 +125,7 @@
     <t>IMPL</t>
   </si>
   <si>
-    <t xml:space="preserve">Spanish - Español para principiantes</t>
+    <t>Spanish - Español para principiantes</t>
   </si>
   <si>
     <t>CONFIRMED</t>
@@ -143,7 +146,7 @@
     <t>ELEM</t>
   </si>
   <si>
-    <t xml:space="preserve">Introduction module</t>
+    <t>Introduction module</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_1_ID</t>
@@ -155,7 +158,7 @@
     <t>MOD</t>
   </si>
   <si>
-    <t xml:space="preserve">Introduction 1</t>
+    <t>Introduction 1</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_1_ID-SC_INTRO_1</t>
@@ -194,7 +197,7 @@
     <t>Zuerich</t>
   </si>
   <si>
-    <t xml:space="preserve">Introduction 2</t>
+    <t>Introduction 2</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_1_ID-SC_INTRO_2</t>
@@ -206,13 +209,13 @@
     <t>P_ESP-IMPL_1_EPP_SP26-M_1_ID-EV_INTRO_2</t>
   </si>
   <si>
-    <t xml:space="preserve">Theory module</t>
+    <t>Theory module</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_2_TH</t>
   </si>
   <si>
-    <t xml:space="preserve">Spanish for beginners - Part 1</t>
+    <t>Spanish for beginners - Part 1</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_2_TH-SC_SFB_P1</t>
@@ -221,7 +224,7 @@
     <t>/LANG/ESP/EPP/TH/</t>
   </si>
   <si>
-    <t xml:space="preserve">Spanish for beginners- Part 1</t>
+    <t>Spanish for beginners- Part 1</t>
   </si>
   <si>
     <t>P_ESP-IMPL_EPP-M_2_TH-TEMP_SFB_P1</t>
@@ -230,22 +233,22 @@
     <t>/LANG/ESP/EPP/TH/;/LOD/LOW/</t>
   </si>
   <si>
-    <t xml:space="preserve">Session 1</t>
+    <t>Session 1</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_2_TH-EV_SFB_P1_1</t>
   </si>
   <si>
-    <t xml:space="preserve">Session 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spanish for beginners - Part 2</t>
+    <t>Session 2</t>
+  </si>
+  <si>
+    <t>Spanish for beginners - Part 2</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_2_TH-SC_SFB_P2</t>
   </si>
   <si>
-    <t xml:space="preserve">Spanish for beginners- Part 2</t>
+    <t>Spanish for beginners- Part 2</t>
   </si>
   <si>
     <t>P_ESP-IMPL_EPP-M_2_TH-TEMP_SFB_P2</t>
@@ -254,7 +257,7 @@
     <t>P_ESP-IMPL_1_EPP_SP26-M_2_TH-EV_SFB_P2_1</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice module</t>
+    <t>Practice module</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_3_PE</t>
@@ -266,7 +269,7 @@
     <t>/LANG/ESP/EPP/PE/</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice 1</t>
+    <t>Practice 1</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_3_PE-CB_PE_1</t>
@@ -278,7 +281,7 @@
     <t>P_ESP-IMPL_1_EPP_SP26-M_3_PE-EV_PE_1</t>
   </si>
   <si>
-    <t xml:space="preserve">Practice 2</t>
+    <t>Practice 2</t>
   </si>
   <si>
     <t>P_ESP-IMPL_1_EPP_SP26-M_3_PE-CB_PE_2</t>
@@ -314,13 +317,13 @@
     <t>P_ESP-IMPL_2_EPP_SU26-M_3_PE</t>
   </si>
   <si>
-    <t xml:space="preserve">Role *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Username *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registration Date</t>
+    <t>Role *</t>
+  </si>
+  <si>
+    <t>Username *</t>
+  </si>
+  <si>
+    <t>Registration Date</t>
   </si>
   <si>
     <t>PARTICIPANT</t>
@@ -359,16 +362,16 @@
     <t>cmueller</t>
   </si>
   <si>
-    <t xml:space="preserve">First Name *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Name *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail *</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORG Affiliation *</t>
+    <t>First Name *</t>
+  </si>
+  <si>
+    <t>Last Name *</t>
+  </si>
+  <si>
+    <t>E-mail *</t>
+  </si>
+  <si>
+    <t>ORG Affiliation *</t>
   </si>
   <si>
     <t>Created</t>
@@ -395,7 +398,7 @@
     <t>UX</t>
   </si>
   <si>
-    <t xml:space="preserve">Marisol Julieta</t>
+    <t>Marisol Julieta</t>
   </si>
   <si>
     <t>De-la-cruz</t>
@@ -455,13 +458,13 @@
     <t>https://testing.frentix.com/test9/</t>
   </si>
   <si>
-    <t xml:space="preserve">OpenOlat Version</t>
+    <t>OpenOlat Version</t>
   </si>
   <si>
     <t>20.2.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Export Language</t>
+    <t>Export Language</t>
   </si>
   <si>
     <t>EN</t>
@@ -470,39 +473,54 @@
     <t>Exported</t>
   </si>
   <si>
-    <t xml:space="preserve">Exported by</t>
+    <t>Exported by</t>
   </si>
   <si>
     <t xml:space="preserve">Faber, Kilian </t>
+  </si>
+  <si>
+    <t>Rooms</t>
+  </si>
+  <si>
+    <t>Zoffice:Meeting-room;Zoffice:Openspace</t>
+  </si>
+  <si>
+    <t>BG_1:AULUA;BG_1:-H101</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="mm&quot;/&quot;dd&quot;/&quot;yyyy&quot;&quot;"/>
     <numFmt numFmtId="165" formatCode="hh:mm&quot; &quot;AM/PM"/>
     <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy&quot; &quot;hh:mm"/>
     <numFmt numFmtId="167" formatCode="mm&quot;/&quot;dd&quot;/&quot;yyyy&quot;, &quot;hh:mm&quot; &quot;AM/PM"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.000000"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
@@ -523,11 +541,11 @@
   </fills>
   <borders count="3">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -542,49 +560,49 @@
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
-      <diagonal style="none"/>
+      <diagonal/>
     </border>
     <border>
-      <left style="none"/>
+      <left/>
       <right style="thin">
         <color rgb="FFB2B2B2"/>
       </right>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="3">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
-    <xf fontId="0" fillId="2" borderId="1" numFmtId="0" applyNumberFormat="0" applyFont="0" applyFill="1" applyBorder="1" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="20">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="2"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="2" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="22" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="166" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="2" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" quotePrefix="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="18" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Notiz" xfId="2" builtinId="10"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="2" builtinId="10"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -599,291 +617,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1094,22 +829,24 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" style="1" width="7.33203125"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" style="1" width="8.83203125"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="1" width="14.33203125"/>
-    <col bestFit="1" customWidth="1" min="4" max="5" width="10.5"/>
-    <col bestFit="1" customWidth="1" min="6" max="6" width="16.1640625"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" width="17.1640625"/>
+    <col min="1" max="1" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="1">
+    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1132,7 +869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1154,41 +891,41 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.78740157500000008" bottom="0.78740157500000008" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157500000008" bottom="0.78740157500000008" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:V78"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="17.5"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" style="1" width="23.5"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" style="1" width="13.83203125"/>
-    <col bestFit="1" customWidth="1" min="4" max="4" style="1" width="7.1640625"/>
-    <col bestFit="1" customWidth="1" min="5" max="5" style="1" width="29.83203125"/>
-    <col bestFit="1" customWidth="1" min="6" max="6" style="1" width="43.6640625"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" width="12.83203125"/>
-    <col bestFit="1" customWidth="1" min="8" max="8" style="5" width="13"/>
-    <col bestFit="1" customWidth="1" min="9" max="9" style="6" width="13.1640625"/>
-    <col bestFit="1" customWidth="1" min="10" max="10" width="11.5"/>
-    <col bestFit="1" customWidth="1" min="11" max="11" style="6" width="11.6640625"/>
-    <col bestFit="1" customWidth="1" min="12" max="12" width="6.1640625"/>
-    <col bestFit="1" customWidth="1" min="13" max="13" width="41.83203125"/>
-    <col bestFit="1" customWidth="1" min="14" max="14" width="10.1640625"/>
-    <col bestFit="1" customWidth="1" min="15" max="15" style="1" width="20.83203125"/>
-    <col bestFit="1" customWidth="1" min="16" max="16" width="10.33203125"/>
-    <col bestFit="1" customWidth="1" min="17" max="17" width="11.1640625"/>
-    <col bestFit="1" customWidth="1" min="18" max="18" width="10.5"/>
-    <col bestFit="1" customWidth="1" min="19" max="19" width="27.1640625"/>
-    <col bestFit="1" customWidth="1" min="20" max="20" style="7" width="18.1640625"/>
-    <col bestFit="1" customWidth="1" min="21" max="21" width="18.1640625"/>
+    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="43.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.1640625" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.1640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="1">
+    <row r="1" spans="1:22" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
@@ -1231,29 +968,32 @@
       <c r="N1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="U1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1281,29 +1021,29 @@
       <c r="J2" s="5">
         <v>46129</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="P2" t="s">
-        <v>35</v>
       </c>
       <c r="Q2" t="s">
         <v>35</v>
       </c>
       <c r="R2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S2" t="s">
         <v>36</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>37</v>
       </c>
-      <c r="T2" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U2" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V2" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1331,29 +1071,29 @@
       <c r="J3" s="5">
         <v>46125</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>36</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>10</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>36</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>37</v>
       </c>
-      <c r="T3" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U3" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V3" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1381,29 +1121,29 @@
       <c r="J4" s="5">
         <v>46125</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>36</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>10</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>36</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>37</v>
       </c>
-      <c r="T4" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U4" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V4" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1425,17 +1165,17 @@
       <c r="G5" t="s">
         <v>48</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>37</v>
       </c>
-      <c r="T5" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U5" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V5" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1463,17 +1203,17 @@
       <c r="J6" s="5">
         <v>46125</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>51</v>
       </c>
-      <c r="T6" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U6" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V6" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1516,17 +1256,20 @@
       <c r="N7" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="S7" t="s">
+      <c r="O7" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="T7" t="s">
         <v>37</v>
       </c>
-      <c r="T7" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U7" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V7" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1554,29 +1297,29 @@
       <c r="J8" s="5">
         <v>46125</v>
       </c>
-      <c r="O8" s="1" t="s">
+      <c r="P8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>36</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
         <v>10</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>36</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>37</v>
       </c>
-      <c r="T8" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U8" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V8" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1598,17 +1341,17 @@
       <c r="G9" t="s">
         <v>48</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>37</v>
       </c>
-      <c r="T9" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U9" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V9" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1636,17 +1379,17 @@
       <c r="J10" s="5">
         <v>46125</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>51</v>
       </c>
-      <c r="T10" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U10" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V10" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1686,17 +1429,20 @@
       <c r="N11" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="S11" t="s">
+      <c r="O11" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="T11" t="s">
         <v>37</v>
       </c>
-      <c r="T11" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U11" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V11" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1724,11 +1470,8 @@
       <c r="J12" s="5">
         <v>46127</v>
       </c>
-      <c r="O12" s="1" t="s">
+      <c r="P12" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="P12" t="s">
-        <v>36</v>
       </c>
       <c r="Q12" t="s">
         <v>36</v>
@@ -1737,16 +1480,19 @@
         <v>36</v>
       </c>
       <c r="S12" t="s">
+        <v>36</v>
+      </c>
+      <c r="T12" t="s">
         <v>37</v>
       </c>
-      <c r="T12" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U12" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V12" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1757,7 +1503,7 @@
         <v>38</v>
       </c>
       <c r="D13" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>62</v>
@@ -1774,11 +1520,8 @@
       <c r="J13" s="5">
         <v>46127</v>
       </c>
-      <c r="O13" s="1" t="s">
+      <c r="P13" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="P13" t="s">
-        <v>36</v>
       </c>
       <c r="Q13" t="s">
         <v>36</v>
@@ -1787,16 +1530,19 @@
         <v>36</v>
       </c>
       <c r="S13" t="s">
+        <v>36</v>
+      </c>
+      <c r="T13" t="s">
         <v>64</v>
       </c>
-      <c r="T13" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U13" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V13" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1807,7 +1553,7 @@
         <v>46</v>
       </c>
       <c r="D14" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>65</v>
@@ -1818,17 +1564,17 @@
       <c r="G14" t="s">
         <v>48</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>64</v>
       </c>
-      <c r="T14" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U14" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V14" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1839,7 +1585,7 @@
         <v>49</v>
       </c>
       <c r="D15" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>65</v>
@@ -1856,17 +1602,17 @@
       <c r="J15" s="5">
         <v>46126</v>
       </c>
-      <c r="S15" t="s">
+      <c r="T15" t="s">
         <v>67</v>
       </c>
-      <c r="T15" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U15" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V15" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1877,7 +1623,7 @@
         <v>52</v>
       </c>
       <c r="D16" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>68</v>
@@ -1904,17 +1650,18 @@
         <v>63</v>
       </c>
       <c r="N16" s="12"/>
-      <c r="S16" t="s">
+      <c r="O16" s="12"/>
+      <c r="T16" t="s">
         <v>64</v>
       </c>
-      <c r="T16" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U16" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V16" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -1925,7 +1672,7 @@
         <v>52</v>
       </c>
       <c r="D17" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>70</v>
@@ -1952,17 +1699,18 @@
         <v>63</v>
       </c>
       <c r="N17" s="12"/>
-      <c r="S17" t="s">
+      <c r="O17" s="12"/>
+      <c r="T17" t="s">
         <v>64</v>
       </c>
-      <c r="T17" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U17" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V17" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1990,11 +1738,8 @@
       <c r="J18" s="5">
         <v>46127</v>
       </c>
-      <c r="O18" s="1" t="s">
+      <c r="P18" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="P18" t="s">
-        <v>36</v>
       </c>
       <c r="Q18" t="s">
         <v>36</v>
@@ -2003,16 +1748,19 @@
         <v>36</v>
       </c>
       <c r="S18" t="s">
+        <v>36</v>
+      </c>
+      <c r="T18" t="s">
         <v>64</v>
       </c>
-      <c r="T18" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U18" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V18" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -2034,17 +1782,17 @@
       <c r="G19" t="s">
         <v>48</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>64</v>
       </c>
-      <c r="T19" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U19" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V19" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -2072,17 +1820,17 @@
       <c r="J20" s="5">
         <v>46127</v>
       </c>
-      <c r="S20" t="s">
+      <c r="T20" t="s">
         <v>67</v>
       </c>
-      <c r="T20" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U20" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V20" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -2120,17 +1868,18 @@
         <v>72</v>
       </c>
       <c r="N21" s="12"/>
-      <c r="S21" t="s">
+      <c r="O21" s="12"/>
+      <c r="T21" t="s">
         <v>64</v>
       </c>
-      <c r="T21" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U21" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V21" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -2168,17 +1917,18 @@
         <v>72</v>
       </c>
       <c r="N22" s="12"/>
-      <c r="S22" t="s">
+      <c r="O22" s="12"/>
+      <c r="T22" t="s">
         <v>64</v>
       </c>
-      <c r="T22" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U22" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V22" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>8</v>
       </c>
@@ -2206,29 +1956,29 @@
       <c r="J23" s="5">
         <v>46129</v>
       </c>
-      <c r="O23" s="1" t="s">
+      <c r="P23" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="P23" t="s">
-        <v>35</v>
       </c>
       <c r="Q23" t="s">
         <v>35</v>
       </c>
       <c r="R23" t="s">
+        <v>35</v>
+      </c>
+      <c r="S23" t="s">
         <v>36</v>
       </c>
-      <c r="S23" t="s">
+      <c r="T23" t="s">
         <v>79</v>
       </c>
-      <c r="T23" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U23" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V23" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>8</v>
       </c>
@@ -2256,17 +2006,17 @@
       <c r="J24" s="5">
         <v>46128</v>
       </c>
-      <c r="S24" t="s">
+      <c r="T24" t="s">
         <v>82</v>
       </c>
-      <c r="T24" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U24" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V24" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -2304,17 +2054,18 @@
         <v>81</v>
       </c>
       <c r="N25" s="12"/>
-      <c r="S25" t="s">
+      <c r="O25" s="12"/>
+      <c r="T25" t="s">
         <v>79</v>
       </c>
-      <c r="T25" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U25" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V25" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -2342,17 +2093,17 @@
       <c r="J26" s="5">
         <v>46129</v>
       </c>
-      <c r="S26" t="s">
+      <c r="T26" t="s">
         <v>82</v>
       </c>
-      <c r="T26" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U26" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V26" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -2390,17 +2141,18 @@
         <v>85</v>
       </c>
       <c r="N27" s="12"/>
-      <c r="S27" t="s">
+      <c r="O27" s="12"/>
+      <c r="T27" t="s">
         <v>79</v>
       </c>
-      <c r="T27" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U27" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V27" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>8</v>
       </c>
@@ -2428,11 +2180,8 @@
       <c r="J28" s="14">
         <v>46213</v>
       </c>
-      <c r="O28" s="1" t="s">
+      <c r="P28" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="P28" t="s">
-        <v>36</v>
       </c>
       <c r="Q28" t="s">
         <v>36</v>
@@ -2441,16 +2190,19 @@
         <v>36</v>
       </c>
       <c r="S28" t="s">
+        <v>36</v>
+      </c>
+      <c r="T28" t="s">
         <v>37</v>
       </c>
-      <c r="T28" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U28" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V28" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>8</v>
       </c>
@@ -2478,29 +2230,29 @@
       <c r="J29" s="14">
         <v>46209</v>
       </c>
-      <c r="O29" s="1" t="s">
+      <c r="P29" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="P29" t="s">
+      <c r="Q29" t="s">
         <v>36</v>
       </c>
-      <c r="Q29" t="s">
+      <c r="R29" t="s">
         <v>10</v>
       </c>
-      <c r="R29" t="s">
+      <c r="S29" t="s">
         <v>36</v>
       </c>
-      <c r="S29" t="s">
+      <c r="T29" t="s">
         <v>37</v>
       </c>
-      <c r="T29" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U29" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V29" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>8</v>
       </c>
@@ -2528,29 +2280,29 @@
       <c r="J30" s="14">
         <v>46209</v>
       </c>
-      <c r="O30" s="1" t="s">
+      <c r="P30" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P30" t="s">
+      <c r="Q30" t="s">
         <v>36</v>
       </c>
-      <c r="Q30" t="s">
+      <c r="R30" t="s">
         <v>10</v>
       </c>
-      <c r="R30" t="s">
+      <c r="S30" t="s">
         <v>36</v>
       </c>
-      <c r="S30" t="s">
+      <c r="T30" t="s">
         <v>37</v>
       </c>
-      <c r="T30" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U30" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V30" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>8</v>
       </c>
@@ -2572,17 +2324,17 @@
       <c r="G31" t="s">
         <v>48</v>
       </c>
-      <c r="S31" t="s">
+      <c r="T31" t="s">
         <v>37</v>
       </c>
-      <c r="T31" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U31" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V31" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>8</v>
       </c>
@@ -2610,29 +2362,29 @@
       <c r="J32" s="14">
         <v>46209</v>
       </c>
-      <c r="O32" s="1" t="s">
+      <c r="P32" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P32" t="s">
+      <c r="Q32" t="s">
         <v>36</v>
       </c>
-      <c r="Q32" t="s">
+      <c r="R32" t="s">
         <v>10</v>
       </c>
-      <c r="R32" t="s">
+      <c r="S32" t="s">
         <v>36</v>
       </c>
-      <c r="S32" t="s">
+      <c r="T32" t="s">
         <v>37</v>
       </c>
-      <c r="T32" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U32" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V32" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -2654,17 +2406,17 @@
       <c r="G33" t="s">
         <v>48</v>
       </c>
-      <c r="S33" t="s">
+      <c r="T33" t="s">
         <v>37</v>
       </c>
-      <c r="T33" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U33" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V33" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -2692,11 +2444,8 @@
       <c r="J34" s="14">
         <v>46211</v>
       </c>
-      <c r="O34" s="1" t="s">
+      <c r="P34" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="P34" t="s">
-        <v>36</v>
       </c>
       <c r="Q34" t="s">
         <v>36</v>
@@ -2705,16 +2454,19 @@
         <v>36</v>
       </c>
       <c r="S34" t="s">
+        <v>36</v>
+      </c>
+      <c r="T34" t="s">
         <v>64</v>
       </c>
-      <c r="T34" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U34" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V34" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -2725,7 +2477,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>62</v>
@@ -2742,11 +2494,8 @@
       <c r="J35" s="14">
         <v>46210</v>
       </c>
-      <c r="O35" s="1" t="s">
+      <c r="P35" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="P35" t="s">
-        <v>36</v>
       </c>
       <c r="Q35" t="s">
         <v>36</v>
@@ -2755,16 +2504,19 @@
         <v>36</v>
       </c>
       <c r="S35" t="s">
+        <v>36</v>
+      </c>
+      <c r="T35" t="s">
         <v>64</v>
       </c>
-      <c r="T35" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U35" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V35" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -2775,7 +2527,7 @@
         <v>46</v>
       </c>
       <c r="D36" s="1">
-        <v>2.1000000000000001</v>
+        <v>2.1</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>65</v>
@@ -2786,17 +2538,17 @@
       <c r="G36" t="s">
         <v>48</v>
       </c>
-      <c r="S36" t="s">
+      <c r="T36" t="s">
         <v>64</v>
       </c>
-      <c r="T36" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U36" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V36" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -2824,11 +2576,8 @@
       <c r="J37" s="14">
         <v>46211</v>
       </c>
-      <c r="O37" s="1" t="s">
+      <c r="P37" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="P37" t="s">
-        <v>36</v>
       </c>
       <c r="Q37" t="s">
         <v>36</v>
@@ -2837,16 +2586,19 @@
         <v>36</v>
       </c>
       <c r="S37" t="s">
+        <v>36</v>
+      </c>
+      <c r="T37" t="s">
         <v>64</v>
       </c>
-      <c r="T37" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U37" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V37" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>8</v>
       </c>
@@ -2868,17 +2620,17 @@
       <c r="G38" t="s">
         <v>48</v>
       </c>
-      <c r="S38" t="s">
+      <c r="T38" t="s">
         <v>64</v>
       </c>
-      <c r="T38" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U38" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V38" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -2906,348 +2658,347 @@
       <c r="J39" s="14">
         <v>46213</v>
       </c>
-      <c r="O39" s="1" t="s">
+      <c r="P39" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="P39" t="s">
-        <v>35</v>
       </c>
       <c r="Q39" t="s">
         <v>35</v>
       </c>
       <c r="R39" t="s">
+        <v>35</v>
+      </c>
+      <c r="S39" t="s">
         <v>36</v>
       </c>
-      <c r="S39" t="s">
+      <c r="T39" t="s">
         <v>79</v>
       </c>
-      <c r="T39" s="11">
-        <v>46034.63958333333</v>
-      </c>
       <c r="U39" s="11">
+        <v>46034.63958333333</v>
+      </c>
+      <c r="V39" s="11">
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="F41" s="15"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E42"/>
       <c r="F42"/>
       <c r="H42"/>
       <c r="I42"/>
       <c r="K42"/>
-      <c r="O42"/>
-    </row>
-    <row r="43">
+      <c r="P42"/>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E43"/>
       <c r="F43"/>
       <c r="H43"/>
       <c r="I43"/>
       <c r="K43"/>
-      <c r="O43"/>
-    </row>
-    <row r="44">
+      <c r="P43"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E44"/>
       <c r="F44"/>
       <c r="H44"/>
       <c r="I44"/>
       <c r="K44"/>
-      <c r="O44"/>
-    </row>
-    <row r="45">
+      <c r="P44"/>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E45"/>
       <c r="F45"/>
       <c r="H45"/>
       <c r="I45"/>
       <c r="K45"/>
-      <c r="O45"/>
-    </row>
-    <row r="46">
+      <c r="P45"/>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E46"/>
       <c r="F46"/>
       <c r="H46"/>
       <c r="I46"/>
       <c r="K46"/>
-      <c r="O46"/>
-    </row>
-    <row r="47">
+      <c r="P46"/>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E47"/>
       <c r="F47"/>
       <c r="H47"/>
       <c r="I47"/>
       <c r="K47"/>
-      <c r="O47"/>
-    </row>
-    <row r="48">
+      <c r="P47"/>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E48"/>
       <c r="F48"/>
       <c r="H48"/>
       <c r="I48"/>
       <c r="K48"/>
-      <c r="O48"/>
-    </row>
-    <row r="49">
+      <c r="P48"/>
+    </row>
+    <row r="49" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E49"/>
       <c r="F49"/>
       <c r="H49"/>
       <c r="I49"/>
       <c r="K49"/>
-      <c r="O49"/>
-    </row>
-    <row r="50">
+      <c r="P49"/>
+    </row>
+    <row r="50" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E50"/>
       <c r="F50"/>
       <c r="H50"/>
       <c r="I50"/>
       <c r="K50"/>
-      <c r="O50"/>
-    </row>
-    <row r="51">
+      <c r="P50"/>
+    </row>
+    <row r="51" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E51"/>
       <c r="F51"/>
       <c r="H51"/>
       <c r="I51"/>
       <c r="K51"/>
-      <c r="O51"/>
-    </row>
-    <row r="52">
+      <c r="P51"/>
+    </row>
+    <row r="52" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E52"/>
       <c r="F52"/>
       <c r="H52"/>
       <c r="I52"/>
       <c r="K52"/>
-      <c r="O52"/>
-    </row>
-    <row r="53">
+      <c r="P52"/>
+    </row>
+    <row r="53" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E53"/>
       <c r="F53"/>
       <c r="H53"/>
       <c r="I53"/>
       <c r="K53"/>
-      <c r="O53"/>
-    </row>
-    <row r="54">
+      <c r="P53"/>
+    </row>
+    <row r="54" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E54"/>
       <c r="F54"/>
       <c r="H54"/>
       <c r="I54"/>
       <c r="K54"/>
-      <c r="O54"/>
-    </row>
-    <row r="55">
+      <c r="P54"/>
+    </row>
+    <row r="55" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E55"/>
       <c r="F55"/>
       <c r="H55"/>
       <c r="I55"/>
       <c r="K55"/>
-      <c r="O55"/>
-    </row>
-    <row r="56">
+      <c r="P55"/>
+    </row>
+    <row r="56" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E56"/>
       <c r="F56"/>
       <c r="H56"/>
       <c r="I56"/>
       <c r="K56"/>
-      <c r="O56"/>
-    </row>
-    <row r="57">
+      <c r="P56"/>
+    </row>
+    <row r="57" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E57"/>
       <c r="F57"/>
       <c r="H57"/>
       <c r="I57"/>
       <c r="K57"/>
-      <c r="O57"/>
-    </row>
-    <row r="58">
+      <c r="P57"/>
+    </row>
+    <row r="58" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E58"/>
       <c r="F58"/>
       <c r="H58"/>
       <c r="I58"/>
       <c r="K58"/>
-      <c r="O58"/>
-    </row>
-    <row r="59">
+      <c r="P58"/>
+    </row>
+    <row r="59" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E59"/>
       <c r="F59"/>
       <c r="H59"/>
       <c r="I59"/>
       <c r="K59"/>
-      <c r="O59"/>
-    </row>
-    <row r="60">
+      <c r="P59"/>
+    </row>
+    <row r="60" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E60"/>
       <c r="F60"/>
       <c r="H60"/>
       <c r="I60"/>
       <c r="K60"/>
-      <c r="O60"/>
-    </row>
-    <row r="61">
+      <c r="P60"/>
+    </row>
+    <row r="61" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E61"/>
       <c r="F61"/>
       <c r="H61"/>
       <c r="I61"/>
       <c r="K61"/>
-      <c r="O61"/>
-    </row>
-    <row r="62">
+      <c r="P61"/>
+    </row>
+    <row r="62" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E62"/>
       <c r="F62"/>
       <c r="H62"/>
       <c r="I62"/>
       <c r="K62"/>
-      <c r="O62"/>
-    </row>
-    <row r="63">
+      <c r="P62"/>
+    </row>
+    <row r="63" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E63"/>
       <c r="F63"/>
       <c r="H63"/>
       <c r="I63"/>
       <c r="K63"/>
-      <c r="O63"/>
-    </row>
-    <row r="64">
+      <c r="P63"/>
+    </row>
+    <row r="64" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E64"/>
       <c r="F64"/>
       <c r="H64"/>
       <c r="I64"/>
       <c r="K64"/>
-      <c r="O64"/>
-    </row>
-    <row r="65">
+      <c r="P64"/>
+    </row>
+    <row r="65" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E65"/>
       <c r="F65"/>
       <c r="H65"/>
       <c r="I65"/>
       <c r="K65"/>
-      <c r="O65"/>
-    </row>
-    <row r="66">
+      <c r="P65"/>
+    </row>
+    <row r="66" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E66"/>
       <c r="F66"/>
       <c r="H66"/>
       <c r="I66"/>
       <c r="K66"/>
-      <c r="O66"/>
-    </row>
-    <row r="67">
+      <c r="P66"/>
+    </row>
+    <row r="67" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E67"/>
       <c r="F67"/>
       <c r="H67"/>
       <c r="I67"/>
       <c r="K67"/>
-      <c r="O67"/>
-    </row>
-    <row r="68">
+      <c r="P67"/>
+    </row>
+    <row r="68" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E68"/>
       <c r="F68"/>
       <c r="H68"/>
       <c r="I68"/>
       <c r="K68"/>
-      <c r="O68"/>
-    </row>
-    <row r="69">
+      <c r="P68"/>
+    </row>
+    <row r="69" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E69"/>
       <c r="F69"/>
       <c r="H69"/>
       <c r="I69"/>
       <c r="K69"/>
-      <c r="O69"/>
-    </row>
-    <row r="70">
+      <c r="P69"/>
+    </row>
+    <row r="70" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E70"/>
       <c r="F70"/>
       <c r="H70"/>
       <c r="I70"/>
       <c r="K70"/>
-      <c r="O70"/>
-    </row>
-    <row r="71">
+      <c r="P70"/>
+    </row>
+    <row r="71" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E71"/>
       <c r="F71"/>
       <c r="H71"/>
       <c r="I71"/>
       <c r="K71"/>
-      <c r="O71"/>
-    </row>
-    <row r="72">
+      <c r="P71"/>
+    </row>
+    <row r="72" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E72"/>
       <c r="F72"/>
       <c r="H72"/>
       <c r="I72"/>
       <c r="K72"/>
-      <c r="O72"/>
-    </row>
-    <row r="73">
+      <c r="P72"/>
+    </row>
+    <row r="73" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E73"/>
       <c r="F73"/>
       <c r="H73"/>
       <c r="I73"/>
       <c r="K73"/>
-      <c r="O73"/>
-    </row>
-    <row r="74">
+      <c r="P73"/>
+    </row>
+    <row r="74" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E74"/>
       <c r="F74"/>
       <c r="H74"/>
       <c r="I74"/>
       <c r="K74"/>
-      <c r="O74"/>
-    </row>
-    <row r="75">
+      <c r="P74"/>
+    </row>
+    <row r="75" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E75"/>
       <c r="F75"/>
       <c r="H75"/>
       <c r="I75"/>
       <c r="K75"/>
-      <c r="O75"/>
-    </row>
-    <row r="76">
+      <c r="P75"/>
+    </row>
+    <row r="76" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E76"/>
       <c r="F76"/>
       <c r="H76"/>
       <c r="I76"/>
       <c r="K76"/>
-      <c r="O76"/>
-    </row>
-    <row r="77">
+      <c r="P76"/>
+    </row>
+    <row r="77" spans="5:16" x14ac:dyDescent="0.2">
       <c r="E77"/>
       <c r="F77"/>
       <c r="H77"/>
       <c r="I77"/>
       <c r="K77"/>
-      <c r="O77"/>
-    </row>
-    <row r="78">
+      <c r="P77"/>
+    </row>
+    <row r="78" spans="5:16" x14ac:dyDescent="0.2">
       <c r="F78"/>
       <c r="H78"/>
       <c r="I78"/>
       <c r="K78"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U39"/>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.78740157500000008" bottom="0.78740157500000008" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
-  <headerFooter/>
+  <autoFilter ref="A1:V39" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157500000008" bottom="0.78740157500000008" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col bestFit="1" min="1" max="1" width="15.5"/>
-    <col bestFit="1" min="2" max="2" width="23.5"/>
-    <col bestFit="1" min="3" max="3" width="41.83203125"/>
-    <col bestFit="1" min="4" max="4" width="16.5"/>
-    <col bestFit="1" min="5" max="5" width="17.5"/>
-    <col bestFit="1" customWidth="1" min="6" max="6" width="18.1640625"/>
-    <col bestFit="1" min="7" max="7" width="18.1640625"/>
+    <col min="1" max="1" width="15.5" bestFit="1"/>
+    <col min="2" max="2" width="23.5" bestFit="1"/>
+    <col min="3" max="3" width="41.83203125" bestFit="1"/>
+    <col min="4" max="4" width="16.5" bestFit="1"/>
+    <col min="5" max="5" width="17.5" bestFit="1"/>
+    <col min="6" max="6" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.1640625" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>13</v>
       </c>
@@ -3270,7 +3021,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -3293,7 +3044,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -3316,7 +3067,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3339,7 +3090,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3362,7 +3113,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -3385,7 +3136,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -3408,7 +3159,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -3431,7 +3182,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -3454,7 +3205,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -3477,7 +3228,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -3500,7 +3251,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -3523,7 +3274,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -3546,7 +3297,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -3569,7 +3320,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -3592,7 +3343,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -3615,7 +3366,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -3638,7 +3389,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -3661,7 +3412,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -3684,7 +3435,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>8</v>
       </c>
@@ -3707,7 +3458,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>8</v>
       </c>
@@ -3730,7 +3481,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -3753,7 +3504,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="17" t="s">
         <v>8</v>
       </c>
@@ -3776,7 +3527,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="17" t="s">
         <v>8</v>
       </c>
@@ -3799,7 +3550,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="17" t="s">
         <v>8</v>
       </c>
@@ -3822,7 +3573,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="17" t="s">
         <v>8</v>
       </c>
@@ -3845,7 +3596,7 @@
         <v>46038.328472222223</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="17" t="s">
         <v>8</v>
       </c>
@@ -3869,26 +3620,25 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="17.5"/>
-    <col bestFit="1" min="2" max="2" width="12.1640625"/>
-    <col bestFit="1" min="3" max="3" width="11.33203125"/>
-    <col bestFit="1" min="4" max="4" width="29.5"/>
-    <col bestFit="1" min="5" max="5" width="14.33203125"/>
-    <col bestFit="1" min="6" max="6" width="18.1640625"/>
+    <col min="1" max="1" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.1640625" bestFit="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1"/>
+    <col min="4" max="4" width="29.5" bestFit="1"/>
+    <col min="5" max="5" width="14.33203125" bestFit="1"/>
+    <col min="6" max="6" width="18.1640625" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>97</v>
       </c>
@@ -3908,7 +3658,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>100</v>
       </c>
@@ -3928,7 +3678,7 @@
         <v>46034.63958333333</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>101</v>
       </c>
@@ -3948,7 +3698,7 @@
         <v>46035.63958333333</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>102</v>
       </c>
@@ -3968,7 +3718,7 @@
         <v>46036.63958333333</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>104</v>
       </c>
@@ -3988,7 +3738,7 @@
         <v>46037.63958333333</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>106</v>
       </c>
@@ -4008,7 +3758,7 @@
         <v>46038.63958333333</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>132</v>
       </c>
@@ -4028,7 +3778,7 @@
         <v>46039.63958333333</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>110</v>
       </c>
@@ -4049,22 +3799,21 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="15.33203125"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" width="24.83203125"/>
+    <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>139</v>
       </c>
@@ -4072,7 +3821,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>141</v>
       </c>
@@ -4080,7 +3829,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>143</v>
       </c>
@@ -4088,7 +3837,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>145</v>
       </c>
@@ -4096,7 +3845,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>147</v>
       </c>
@@ -4104,7 +3853,7 @@
         <v>46038.709027777775</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>148</v>
       </c>
@@ -4114,11 +3863,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B2"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
   </hyperlinks>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.78740157500000008" bottom="0.78740157500000008" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157500000008" bottom="0.78740157500000008" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>